<commit_message>
implement complete weighing machine application
- Added weighing machine application layer
- Integrated ADC driver with internal temperature sensor
- Added moving average filter for stable ADC readings
- Implemented zero calibration using PA0 push button
- Added calibration module for relative value calculation
- Added GPIO_ReadPin() API for button handling
- Integrated ADC, filter and calibration into application
- Verified complete end-to-end application workflow
- Added functional validation and test evidence
</commit_message>
<xml_diff>
--- a/Validation/STM32_Weighing_Machine_Validation.xlsx
+++ b/Validation/STM32_Weighing_Machine_Validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\stm32-project-02-weighing-machine\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C702477-1764-452D-97EE-5BA5275B9FD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AC9B674-B831-4724-A540-F0E6874EF878}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project_Info" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="182">
   <si>
     <t>Field</t>
   </si>
@@ -167,48 +167,6 @@
   </si>
   <si>
     <t>Description</t>
-  </si>
-  <si>
-    <t>Expected</t>
-  </si>
-  <si>
-    <t>Actual</t>
-  </si>
-  <si>
-    <t>WM-001</t>
-  </si>
-  <si>
-    <t>Power On</t>
-  </si>
-  <si>
-    <t>Display initializes</t>
-  </si>
-  <si>
-    <t>WM-002</t>
-  </si>
-  <si>
-    <t>Zero Weight</t>
-  </si>
-  <si>
-    <t>0 Kg displayed</t>
-  </si>
-  <si>
-    <t>WM-003</t>
-  </si>
-  <si>
-    <t>1 Kg Load</t>
-  </si>
-  <si>
-    <t>1 Kg ± tolerance</t>
-  </si>
-  <si>
-    <t>WM-004</t>
-  </si>
-  <si>
-    <t>5 Kg Load</t>
-  </si>
-  <si>
-    <t>5 Kg ± tolerance</t>
   </si>
   <si>
     <t>Defect ID</t>
@@ -646,6 +604,167 @@
   </si>
   <si>
     <t>random values in DR</t>
+  </si>
+  <si>
+    <t>Objective</t>
+  </si>
+  <si>
+    <t>APP-001</t>
+  </si>
+  <si>
+    <t>Application Initialization</t>
+  </si>
+  <si>
+    <t>Weighing machine application shall initialize ADC, Moving Average Filter and Calibration module before operation.</t>
+  </si>
+  <si>
+    <t>Verify successful application initialization.</t>
+  </si>
+  <si>
+    <t>ADC initialized, filter initialized and calibration initialized successfully.</t>
+  </si>
+  <si>
+    <t>APP-001_Initialization.png</t>
+  </si>
+  <si>
+    <t>APP-002</t>
+  </si>
+  <si>
+    <t>Zero Calibration</t>
+  </si>
+  <si>
+    <t>Application shall set the current filtered ADC value as zero reference when PA0 button is pressed.</t>
+  </si>
+  <si>
+    <t>Verify zero calibration.</t>
+  </si>
+  <si>
+    <t>Application initialized and ADC conversions running.</t>
+  </si>
+  <si>
+    <t>Current filtered ADC value stored as zero reference. Measured value becomes approximately 0.</t>
+  </si>
+  <si>
+    <t>Measured value becomes approximately 0.</t>
+  </si>
+  <si>
+    <t>APP-002_Zero_Calibration.png</t>
+  </si>
+  <si>
+    <t>APP-003</t>
+  </si>
+  <si>
+    <t>Continuous Measurement</t>
+  </si>
+  <si>
+    <t>Application shall continuously acquire and process ADC samples.</t>
+  </si>
+  <si>
+    <t>Verify continuous measurement.</t>
+  </si>
+  <si>
+    <t>Application running.</t>
+  </si>
+  <si>
+    <t>Measured value updates continuously according to temperature changes.</t>
+  </si>
+  <si>
+    <t>Value updated continuously.</t>
+  </si>
+  <si>
+    <t>APP-003_Continuous_Measurement.png</t>
+  </si>
+  <si>
+    <t>APP-004</t>
+  </si>
+  <si>
+    <t>Moving Average Filter</t>
+  </si>
+  <si>
+    <t>Application shall filter raw ADC samples before calculating output value.</t>
+  </si>
+  <si>
+    <t>Verify moving average filter integration.</t>
+  </si>
+  <si>
+    <t>Filtered value is smoother and less noisy than raw ADC value.</t>
+  </si>
+  <si>
+    <t>Filtered value smoother than raw ADC value.</t>
+  </si>
+  <si>
+    <t>APP-004_Moving_Average.png</t>
+  </si>
+  <si>
+    <t>APP-005</t>
+  </si>
+  <si>
+    <t>Relative Value Calculation</t>
+  </si>
+  <si>
+    <t>Application shall calculate output relative to calibrated zero reference.</t>
+  </si>
+  <si>
+    <t>Verify calibration algorithm.</t>
+  </si>
+  <si>
+    <t>Zero calibration completed.</t>
+  </si>
+  <si>
+    <t>Output changes relative to zero reference instead of absolute ADC value.</t>
+  </si>
+  <si>
+    <t>Relative value calculated correctly.</t>
+  </si>
+  <si>
+    <t>APP-005_Relative_Value.png</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Call </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>WeighingMachine_Init()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. 
+2. Pause execution after initialization. 
+3. Verify ADC is enabled and conversions are running. 
+4. Verify filter and calibration structures are initialized.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Observe current value. 
+2. Press PA0 button. 
+3. Release button. 
+4. Verify zero offset is updated.</t>
+  </si>
+  <si>
+    <t>1. Run application. 
+2. Observe measured value in Live Expressions/Watch Window. 
+3. Warm the MCU using finger.</t>
+  </si>
+  <si>
+    <t>1. Observe raw ADC value. 
+2. Observe filtered value. 
+3. Compare both values while changing temperature.</t>
+  </si>
+  <si>
+    <t>1. Perform zero calibration. 
+2. Change MCU temperature. 
+3. Observe calculated output.</t>
   </si>
 </sst>
 </file>
@@ -735,14 +854,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1103,7 +1222,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8092B03-5892-4ED1-BFFE-9827AA5F27F3}">
-  <dimension ref="A2:L14"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="4" width="17.33203125" customWidth="1"/>
@@ -1115,446 +1234,446 @@
     <col min="11" max="11" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:12">
-      <c r="A2" s="1" t="s">
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="72">
+      <c r="A2" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="K2" s="8"/>
+      <c r="L2" s="10"/>
+    </row>
+    <row r="3" spans="1:12" ht="72">
+      <c r="A3" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E3" t="s">
         <v>72</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="F3" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="G3" t="s">
         <v>74</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H3" t="s">
+        <v>74</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="J3" t="s">
         <v>75</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="72">
-      <c r="A3" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="K3" s="8"/>
       <c r="L3" s="10"/>
     </row>
-    <row r="4" spans="1:12" ht="72">
-      <c r="A4" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="D4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" t="s">
-        <v>88</v>
-      </c>
-      <c r="H4" t="s">
-        <v>88</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="J4" t="s">
-        <v>89</v>
-      </c>
-      <c r="K4" s="8"/>
+    <row r="4" spans="1:12" ht="57.6">
+      <c r="A4" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K4" s="2"/>
       <c r="L4" s="10"/>
     </row>
     <row r="5" spans="1:12" ht="57.6">
       <c r="A5" s="11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>129</v>
+        <v>78</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>114</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="K5" s="2"/>
       <c r="L5" s="10"/>
     </row>
     <row r="6" spans="1:12" ht="57.6">
       <c r="A6" s="11" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>128</v>
+        <v>78</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>122</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="10"/>
     </row>
     <row r="7" spans="1:12" ht="57.6">
       <c r="A7" s="11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="E7" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="10"/>
     </row>
     <row r="8" spans="1:12" ht="57.6">
       <c r="A8" s="11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>137</v>
+        <v>78</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>124</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="10"/>
     </row>
     <row r="9" spans="1:12" ht="57.6">
       <c r="A9" s="11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>138</v>
+        <v>78</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>125</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="K9" s="2"/>
       <c r="L9" s="10"/>
     </row>
-    <row r="10" spans="1:12" ht="57.6">
+    <row r="10" spans="1:12" ht="72">
       <c r="A10" s="11" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>139</v>
+        <v>78</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>126</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="K10" s="2"/>
       <c r="L10" s="10"/>
     </row>
     <row r="11" spans="1:12" ht="72">
       <c r="A11" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>140</v>
+        <v>78</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>127</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="K11" s="2"/>
       <c r="L11" s="10"/>
     </row>
-    <row r="12" spans="1:12" ht="72">
+    <row r="12" spans="1:12" ht="57.6">
       <c r="A12" s="11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>141</v>
+        <v>111</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>151</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="H12" s="2"/>
       <c r="I12" s="2" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="K12" s="2"/>
       <c r="L12" s="10"/>
     </row>
-    <row r="13" spans="1:12" ht="57.6">
-      <c r="A13" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="H13" s="2"/>
+    <row r="13" spans="1:12" ht="100.8">
+      <c r="A13" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>138</v>
+      </c>
       <c r="I13" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="K13" s="2"/>
-      <c r="L13" s="10"/>
-    </row>
-    <row r="14" spans="1:12" ht="100.8">
-      <c r="A14" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="J14" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="K14" s="8" t="s">
-        <v>135</v>
+        <v>68</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -1566,81 +1685,219 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{725D907A-55B4-4E0D-AF3B-2D945273D0E6}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="13.6640625" customWidth="1"/>
-    <col min="3" max="3" width="16.77734375" customWidth="1"/>
+    <col min="1" max="1" width="13.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.77734375" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" customWidth="1"/>
+    <col min="5" max="5" width="14.44140625" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" customWidth="1"/>
+    <col min="7" max="7" width="19" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="10" max="10" width="23.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>47</v>
+        <v>139</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="J1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="100.8">
       <c r="A2" s="2" t="s">
-        <v>48</v>
+        <v>140</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>49</v>
+        <v>141</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5">
+        <v>142</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="K2" s="2"/>
+    </row>
+    <row r="3" spans="1:11" ht="86.4">
       <c r="A3" s="2" t="s">
-        <v>51</v>
+        <v>146</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>52</v>
+        <v>147</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="4" spans="1:5">
+        <v>148</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="K3" s="2"/>
+    </row>
+    <row r="4" spans="1:11" ht="72">
       <c r="A4" s="2" t="s">
-        <v>54</v>
+        <v>154</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>55</v>
+        <v>155</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5">
+        <v>156</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="K4" s="2"/>
+    </row>
+    <row r="5" spans="1:11" ht="72">
       <c r="A5" s="2" t="s">
-        <v>57</v>
+        <v>162</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>58</v>
+        <v>163</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+        <v>164</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="K5" s="2"/>
+    </row>
+    <row r="6" spans="1:11" ht="72">
+      <c r="A6" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="K6" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1657,19 +1914,19 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28.8">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>19</v>
@@ -1677,7 +1934,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1700,47 +1957,71 @@
   <sheetData>
     <row r="1" spans="1:5" ht="28.8">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>39</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+        <v>55</v>
+      </c>
+      <c r="B2" s="2">
+        <v>12</v>
+      </c>
+      <c r="C2" s="2">
+        <v>12</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="E2" s="14">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="B3" s="2">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0</v>
+      </c>
+      <c r="E3" s="14">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+        <v>57</v>
+      </c>
+      <c r="B4" s="2">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2">
+        <v>17</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+      <c r="E4" s="14">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>